<commit_message>
updated total pigment figure
</commit_message>
<xml_diff>
--- a/data/frag_data/Surface_Area.xlsx
+++ b/data/frag_data/Surface_Area.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://olddominion-my.sharepoint.com/personal/dbarshis_odu_edu/Documents/BarshisLab/FieldWork/2023_034567_AmSamoa/Katie's_Stuff/Respirometry Runs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2917054de0bc48a0/Documents/Barshis_Lab/Field_Work/2023-March-April_American-Samoa/data/frag_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="69" documentId="8_{D37593F5-BBAC-4797-8CAE-41473A31C395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D05E35CF-0717-403D-B1D2-795138A925B8}"/>
+  <xr:revisionPtr revIDLastSave="72" documentId="8_{D37593F5-BBAC-4797-8CAE-41473A31C395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F1ED5D1-080A-404F-8D6D-7DD90D9CA37E}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{9021C3D7-74DC-4965-ADF5-F50A19582A88}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{9021C3D7-74DC-4965-ADF5-F50A19582A88}"/>
   </bookViews>
   <sheets>
     <sheet name="MasterSheet" sheetId="2" r:id="rId1"/>
@@ -514,14 +514,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{695A72CA-5C65-40AB-91E7-BF50853B35EC}">
   <dimension ref="A1:B20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.85546875" customWidth="1"/>
-    <col min="2" max="2" width="23.42578125" customWidth="1"/>
-    <col min="3" max="3" width="18.140625" customWidth="1"/>
+    <col min="1" max="1" width="14.81640625" customWidth="1"/>
+    <col min="2" max="2" width="23.453125" customWidth="1"/>
+    <col min="3" max="3" width="18.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -529,7 +529,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -537,7 +537,7 @@
         <v>24.784747847478474</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -545,7 +545,7 @@
         <v>15.179669653839396</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -553,7 +553,7 @@
         <v>15.610173958882445</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -561,7 +561,7 @@
         <v>16.012124406958357</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -569,7 +569,7 @@
         <v>16.007731505886486</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -577,7 +577,7 @@
         <v>20.040414689861183</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -585,7 +585,7 @@
         <v>24.791337199086275</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -593,7 +593,7 @@
         <v>22.206114918292037</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -601,7 +601,7 @@
         <v>25.654542259708311</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -609,7 +609,7 @@
         <v>24.912141978562644</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -617,7 +617,7 @@
         <v>20.826743981725532</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -625,7 +625,7 @@
         <v>16.071428571428569</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -633,7 +633,7 @@
         <v>22.476278334211916</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -641,7 +641,7 @@
         <v>24.48603057459146</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -649,7 +649,7 @@
         <v>14.889738183096117</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -657,7 +657,7 @@
         <v>22.22807942365138</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -665,7 +665,7 @@
         <v>25.294324371815147</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -673,7 +673,7 @@
         <v>18.516078017923036</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -690,16 +690,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBB55095-6167-4A6A-9415-7C3572732834}">
   <dimension ref="A1:F28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="20.42578125" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" customWidth="1"/>
+    <col min="3" max="3" width="19.26953125" customWidth="1"/>
+    <col min="4" max="4" width="20.453125" customWidth="1"/>
+    <col min="5" max="5" width="13.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -713,7 +713,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -735,7 +735,7 @@
         <v>4.5528000000000001E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -757,7 +757,7 @@
         <v>3.0114559048185644E-5</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -772,7 +772,7 @@
         <v>4.5111999999999999E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -783,7 +783,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -795,7 +795,7 @@
         <v>24.784747847478474</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -807,7 +807,7 @@
         <v>15.179669653839396</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -819,7 +819,7 @@
         <v>15.610173958882445</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -831,7 +831,7 @@
         <v>16.012124406958357</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -843,7 +843,7 @@
         <v>16.007731505886486</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -855,7 +855,7 @@
         <v>20.040414689861183</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -867,7 +867,7 @@
         <v>24.791337199086275</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -879,7 +879,7 @@
         <v>22.206114918292037</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>12</v>
       </c>
@@ -891,7 +891,7 @@
         <v>25.654542259708311</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -903,7 +903,7 @@
         <v>24.912141978562644</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -915,7 +915,7 @@
         <v>20.826743981725532</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>14</v>
       </c>
@@ -927,7 +927,7 @@
         <v>16.071428571428569</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -939,7 +939,7 @@
         <v>22.476278334211916</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>18</v>
       </c>
@@ -951,7 +951,7 @@
         <v>24.48603057459146</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -963,7 +963,7 @@
         <v>14.889738183096117</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>20</v>
       </c>
@@ -975,7 +975,7 @@
         <v>22.22807942365138</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -987,7 +987,7 @@
         <v>25.294324371815147</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>21</v>
       </c>
@@ -999,7 +999,7 @@
         <v>18.516078017923036</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>19</v>
       </c>
@@ -1011,7 +1011,7 @@
         <v>32.322966086803724</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B27" s="1" t="s">
         <v>27</v>
       </c>
@@ -1020,7 +1020,7 @@
         <v>21.174245577042232</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B28" s="1" t="s">
         <v>29</v>
       </c>

</xml_diff>